<commit_message>
feat(strategy): add iPhone to curated stock and prioritize iPhone in comment bot
</commit_message>
<xml_diff>
--- a/affiliate_data/rocket_curated.xlsx
+++ b/affiliate_data/rocket_curated.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1733,6 +1733,106 @@
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztn-msxxsasoiscl48</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>48900.00</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8AWCoHKL6C</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Apple iPhone 17 Pro (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztf-msuyb0tv79qff4</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>39900.00</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5AsbEphgh5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Apple iPhone 16 Plus (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztg-msuy0uk4gkjo7b</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>34900.00</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/LnLTzHQeV</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Apple iPhone 15 (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://store.storeimages.cdn-apple.com/8756/as-images.apple.com/is/iphone-15-finish-select-202309-6-1inch-black?wid=5120&amp;hei=2880&amp;fmt=p-jpg&amp;qlt=80&amp;.v=1692923777972</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>26900.00</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8fSTPKxXrZ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>